<commit_message>
GSB 784c86e6-484b-5a0e-a7a2-6b3afdb98348 A: platform archive
</commit_message>
<xml_diff>
--- a/samples/sample_impact.xlsx
+++ b/samples/sample_impact.xlsx
@@ -14,7 +14,8 @@
     <sheet name="循环" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="数据" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="审计示例" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="名称" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="关键节点" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="名称" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="单价">参数!$B$2</definedName>
@@ -32,7 +33,7 @@
     <definedName name="环甲">环乙</definedName>
     <definedName name="环乙">环甲</definedName>
     <definedName name="系数" localSheetId="1">参数!$B$4</definedName>
-    <definedName name="折扣" localSheetId="7">参数!$B$4</definedName>
+    <definedName name="折扣" localSheetId="8">参数!$B$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2501,6 +2502,165 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>收入渠道1</t>
+        </is>
+      </c>
+      <c r="B1" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>收入渠道2</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>成本项1</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>成本项2</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>收入合计（关键汇聚点）</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>B1+B2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>成本合计（关键汇聚点）</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>B3+B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>毛利（目标单元格示例）</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>B6-B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>渠道分成1（收入侧旁路）</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>B1*0.1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>渠道分成2（收入侧旁路）</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>B2*0.1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>分成合计（次要汇聚点）</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>B10+B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>净利（目标单元格示例）</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>B8-B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>循环示例（SCC 压缩演示）</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>B16+1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16">
+        <f>B15+B2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>受循环影响的目标</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>B15*2</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>